<commit_message>
Sprint3 execution log (#40)
* Delete sprint3/execution-log.xlsx

deleting the outdated table

* adding the updated version of execution-log.xlsx

update execution log according to review requirements

* Update README.md
</commit_message>
<xml_diff>
--- a/sprint3/execution-log.xlsx
+++ b/sprint3/execution-log.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Environment" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Run 1'!$A$4:$H$54</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Environment'!$A$4:$B$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Run 1'!$A$4:$K$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Environment'!$A$4:$B$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,23 +455,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H54"/>
+  <dimension ref="A1:K78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="90" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="90" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Журнал виконання тест-кейсів — Run 1</t>
+          <t>Журнал виконання тест-кейсів — Run 1 (рядок = одне виконання; зараховано останнє виконання кейсу)</t>
         </is>
       </c>
     </row>
@@ -490,35 +493,50 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
+          <t>Прохід</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
           <t>TC-ID</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Дата</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Час</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Виконавець</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Середовище</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Статус</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Зараховано</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Коментар</t>
         </is>
@@ -532,33 +550,48 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
           <t>TC-001</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>Dashboard; меню з 12 пунктів: Admin, PIM, Leave, Time, Recruitment, My Info, Performance, Dashboard, Directory, Maintenance, Claim, Buzz.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: перелік пунктів меню на кроці 3 не записано, результат не підтверджено.</t>
         </is>
       </c>
     </row>
@@ -570,31 +603,46 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
           <t>TC-002</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr"/>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>«Invalid credentials» лишається після повторного введення Username; вхід із правильним паролем успішний.</t>
         </is>
@@ -608,31 +656,46 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
           <t>TC-003</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
         <is>
           <t>«Account disabled» для qp.ess.off; Dashboard не відкрито.</t>
         </is>
@@ -646,31 +709,46 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
           <t>TC-004</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
         <is>
           <t>Логотип, «Login», панель Admin / admin123, «Forgot your password?»; заповнювачі Username / Password; пароль маскується.</t>
         </is>
@@ -684,35 +762,50 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
           <t>TC-005</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
         <is>
           <t>failed (крок 2)</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>BUG-001 (#23)</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="J9" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
         <is>
           <t>Біля назв Username і Password немає «*»; «Required» на кроці 3 — як очікувано.</t>
         </is>
@@ -726,31 +819,46 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
           <t>TC-006</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr"/>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
         <is>
           <t>12 пунктів меню; пошук «Lea» лишає Leave; меню користувача About, Support, Change Password, Logout.</t>
         </is>
@@ -764,31 +872,46 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
           <t>TC-007</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>13:54</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr"/>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
         <is>
           <t>Після Logout пряма адреса pim/viewEmployeeList переадресовує на /auth/login.</t>
         </is>
@@ -802,37 +925,52 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
           <t>TC-008</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>15:17</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>failed (крок 5)</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="I12" s="4" t="inlineStr">
         <is>
           <t>BUG-002 (#24)</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t>Після 16 хв 19 с бездіяльності (20:46:28–21:02:47) Leave List відкрився без входу. Відтворено у двох сеансах.</t>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: відтворюваність записано без повторного 16-хвилинного очікування.</t>
         </is>
       </c>
     </row>
@@ -844,31 +982,46 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
           <t>TC-009</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F13" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
         <is>
           <t>qp5us створено: «(1) Record Found», ESS, Qpivan Testenko, Enabled; видалено очищенням.</t>
         </is>
@@ -882,31 +1035,46 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
           <t>TC-010</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr"/>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
         <is>
           <t>«Should be at least 5 characters»; форма не збережена.</t>
         </is>
@@ -920,31 +1088,46 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
           <t>TC-011</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>14:14</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
         <is>
           <t>Ім'я з 40 символів збережено; видалено очищенням.</t>
         </is>
@@ -958,31 +1141,46 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
           <t>TC-012</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
         <is>
           <t>«Should not exceed 40 characters»; форма не збережена.</t>
         </is>
@@ -996,31 +1194,46 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
           <t>TC-013</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr"/>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
         <is>
           <t>«Already exists»; форма не збережена.</t>
         </is>
@@ -1034,37 +1247,52 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
           <t>TC-014</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F18" s="4" t="inlineStr">
-        <is>
-          <t>failed (крок 9)</t>
-        </is>
-      </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H18" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 6)</t>
+        </is>
+      </c>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
           <t>BUG-003 (#25)</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
-        <is>
-          <t>Повідомлення про 8 символів немає (індикатор «Better»); на кроці 10 користувача збережено і видалено очищенням.</t>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: номер кроку не збігся з кейсом (6 замість 9), крок 10 (чи збережено користувача) не перевірено.</t>
         </is>
       </c>
     </row>
@@ -1076,37 +1304,52 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
           <t>TC-015</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F19" s="4" t="inlineStr">
-        <is>
-          <t>failed (крок 9)</t>
-        </is>
-      </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 6)</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
           <t>BUG-004 (#26)</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
-        <is>
-          <t>Повідомлення про велику літеру немає (індикатор «Strong»); користувача збережено і видалено очищенням.</t>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: номер кроку не збігся з кейсом (6 замість 9), крок 10 (чи збережено користувача) не перевірено.</t>
         </is>
       </c>
     </row>
@@ -1118,37 +1361,52 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
           <t>TC-016</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>13:57</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>failed (крок 9)</t>
-        </is>
-      </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 6)</t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
           <t>BUG-005 (#27)</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>Повідомлення про спецсимвол немає (індикатор «Weak»); користувача збережено і видалено очищенням.</t>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: номер кроку не збігся з кейсом (6 замість 9), крок 10 (чи збережено користувача) не перевірено.</t>
         </is>
       </c>
     </row>
@@ -1160,31 +1418,46 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
           <t>TC-017</t>
         </is>
       </c>
-      <c r="C21" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>13:58</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F21" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr"/>
+      <c r="J21" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
         <is>
           <t>«Passwords do not match»; форма не збережена.</t>
         </is>
@@ -1198,33 +1471,48 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
           <t>TC-018</t>
         </is>
       </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
           <t>Мініцька А.</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Стовпці і фільтри за F-40; Include: Current Employees Only / Current and Past Employees / Past Employees Only; пошук за Id — (1) Record Found.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr"/>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: варіанти списку Include на кроці 5 не записано.</t>
         </is>
       </c>
     </row>
@@ -1236,31 +1524,46 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
           <t>TC-019</t>
         </is>
       </c>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
           <t>Мініцька А.</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F23" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr"/>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
         <is>
           <t>«(143) Records Found»; прапорець, кошик, олівець у рядку; сортування Last Name в обидва боки.</t>
         </is>
@@ -1274,31 +1577,46 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
           <t>TC-020</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
           <t>Мініцька А.</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr"/>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
         <is>
           <t>1280×720: горизонтальної прокрутки немає (scrollWidth = clientWidth = 886), видно всі стовпці й Actions.</t>
         </is>
@@ -1312,37 +1630,48 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
           <t>TC-021</t>
         </is>
       </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
           <t>Мініцька А.</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F25" s="4" t="inlineStr">
-        <is>
-          <t>failed (крок 7)</t>
-        </is>
-      </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>BUG-006 (#28)</t>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t>«Success / Successfully Saved» ліворуч унизу замість праворуч; запропонований Employee Id записано; Qpanna видалено.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr"/>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: текст і розташування тоста на кроці 7 не перевірено.</t>
         </is>
       </c>
     </row>
@@ -1354,31 +1683,46 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
           <t>TC-022</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>14:23</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
           <t>Мініцька А.</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr"/>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
         <is>
           <t>«Required» під First Name і Last Name; форма не збережена; зірочка біля Employee Full Name є.</t>
         </is>
@@ -1392,31 +1736,46 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
           <t>TC-023</t>
         </is>
       </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
           <t>Мініцька А.</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr"/>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
         <is>
           <t>«Employee Id already exists»; працівника не створено.</t>
         </is>
@@ -1430,35 +1789,50 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
           <t>TC-024</t>
         </is>
       </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>14:23</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
           <t>Мініцька А.</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>failed (крок 6)</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="I28" s="4" t="inlineStr">
         <is>
           <t>BUG-006 (#28)</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
         <is>
           <t>«Successfully Updated» ліворуч унизу замість праворуч; Other Id = QP-OTHER-01 збережено.</t>
         </is>
@@ -1472,35 +1846,50 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
           <t>TC-025</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
           <t>Мініцька А.</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
         <is>
           <t>failed (крок 4)</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="I29" s="4" t="inlineStr">
         <is>
           <t>BUG-007 (#29)</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
         <is>
           <t>Поле First Name доступне для введення, є кнопка Save (дані не зберігались).</t>
         </is>
@@ -1514,37 +1903,48 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
           <t>TC-026</t>
         </is>
       </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>Шпилька Т.</t>
+          <t>27.10.2026</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+          <t>14:19</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>failed (крок 7)</t>
+          <t>Мініцька А.</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>BUG-008 (#31)</t>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>p95 = 6,48 с (10 з 20 &gt; 3 с). Відхилення: 4-та сторінка — Admin → User Management замість Recruitment → Vacancies (без неї 7 з 15 &gt; 3 с); швидкість каналу виміряно не перед замірами, а 28.10.2026 з того самого підключення: fast.com — 910 Мбіт/с (≥ 10 за передумовою).</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr"/>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: час виміряно не за кроками кейсу (не значення Finish у DevTools → Network).</t>
         </is>
       </c>
     </row>
@@ -1556,31 +1956,46 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
           <t>TC-027</t>
         </is>
       </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr"/>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
         <is>
           <t>Ліміт 2.50 для US - Personal збережено («Successfully Saved») і видалено.</t>
         </is>
@@ -1594,31 +2009,46 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
           <t>TC-028</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>14:55</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr"/>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
         <is>
           <t>«Should be a number with upto 2 decimal places»; ліміт не збережено.</t>
         </is>
@@ -1632,33 +2062,52 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
           <t>TC-029</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
-        <is>
-          <t>28.10.2026</t>
-        </is>
-      </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>14:53</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H33" s="4" t="inlineStr">
         <is>
-          <t>Виконано за версією кейсу 1.1 (прохід 3): після введення дат показано список Partial Days. Версія 1.0 у проході 2 дала хибний failed через помилку в очікуваному (аркуш Review).</t>
+          <t>failed (крок 3)</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>— (дефект кейсу)</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: кроки виконано не за нумерацією кейсу (failed на кроці 3); очікуване версії 1.0 щодо Partial Days не випливає з GUI-70 — дефект тест-кейсу, баг-репорт не заводиться.</t>
         </is>
       </c>
     </row>
@@ -1670,31 +2119,46 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
           <t>TC-030</t>
         </is>
       </c>
-      <c r="C34" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G34" s="4" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr"/>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
         <is>
           <t>Пт 20.11 – пн 23.11 = 2.00 дні; Pending Approval (2.00); баланс 3.00; заявку скасовано.</t>
         </is>
@@ -1708,37 +2172,48 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
           <t>TC-031</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>failed (крок 8)</t>
-        </is>
-      </c>
       <c r="G35" s="4" t="inlineStr">
         <is>
-          <t>BUG-009 (#32)</t>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
         </is>
       </c>
       <c r="H35" s="4" t="inlineStr">
         <is>
-          <t>Number of Days 3.00 замість 5.00 — свята 11.11 і 12.11 вилучено. Заявку скасовано.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: очікуване переписано під фактичне (3.00 замість 5.00 з кейсу), тому статус passed хибний.</t>
         </is>
       </c>
     </row>
@@ -1750,31 +2225,46 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
           <t>TC-032</t>
         </is>
       </c>
-      <c r="C36" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>14:54</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G36" s="4" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H36" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I36" s="4" t="inlineStr"/>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
         <is>
           <t>«To date should be after from date»; заявку не подано.</t>
         </is>
@@ -1788,33 +2278,48 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
           <t>TC-033</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H37" s="4" t="inlineStr">
         <is>
-          <t>«Balance not sufficient»; після Apply тост «Leave Balance Exceeded»; заявки немає в My Leave.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr"/>
+      <c r="J37" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K37" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: дати 2026-23-11 – 2026-30-11 замість 2026-16-11 – 2026-23-11 з кейсу.</t>
         </is>
       </c>
     </row>
@@ -1826,33 +2331,48 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
           <t>TC-034</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>16–20.11 = 5.00 при балансі 5.00: «Successfully Saved», Pending Approval (5.00); скасовано.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr"/>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: дати 2026-23-11 – 2026-27-11 замість 2026-16-11 – 2026-20-11 з кейсу.</t>
         </is>
       </c>
     </row>
@@ -1864,33 +2384,48 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
           <t>TC-035</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H39" s="4" t="inlineStr">
         <is>
-          <t>Заявку 17.11 скасовано: Cancelled (1.00), баланс знову 5.00; фільтр статусів — 5 варіантів.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: дата 2026-24-11 замість 2026-17-11 з кейсу.</t>
         </is>
       </c>
     </row>
@@ -1902,33 +2437,48 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
           <t>TC-036</t>
         </is>
       </c>
-      <c r="C40" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>14:58</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G40" s="4" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Заявка 18.11 відхилена Admin: Rejected (1.00), кнопки Cancel у ESS немає.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr"/>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: дата 2026-25-11 замість 2026-18-11 з кейсу.</t>
         </is>
       </c>
     </row>
@@ -1940,33 +2490,48 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
           <t>TC-037</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H41" s="4" t="inlineStr">
         <is>
-          <t>My Actions «(1) Leave Requests to Approve»; Approve → Scheduled (1.00); скасовано очищенням.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr"/>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: дата 2026-26-11 замість 2026-19-11 з кейсу.</t>
         </is>
       </c>
     </row>
@@ -1978,31 +2543,46 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
           <t>TC-038</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H42" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr"/>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
         <is>
           <t>Assign Leave 24.11: «Successfully Saved», Scheduled (1.00); скасовано.</t>
         </is>
@@ -2016,31 +2596,46 @@
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
           <t>TC-039</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
           <t>Любочка В.</t>
         </is>
       </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr"/>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
         <is>
           <t>Діалог «Confirm Leave Assignment … does not have sufficient leave balance…»; Cancel — відпустку не призначено.</t>
         </is>
@@ -2054,33 +2649,48 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
           <t>TC-040</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Табель 26.10–01.11, ACME Ltd / Bug Fixes, 8:00: Save → Not Submitted, Submit → Submitted.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I44" s="4" t="inlineStr"/>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: активність Administration замість Bug Fixes з кейсу.</t>
         </is>
       </c>
     </row>
@@ -2092,33 +2702,48 @@
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
           <t>TC-041</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H45" s="4" t="inlineStr">
         <is>
-          <t>Табель 19.10–25.10 подано (Submitted) і затверджено Admin з коментарем QP TC-041 (Approved).</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr"/>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: тиждень 26.10–01.11 замість 19.10–25.10 з кейсу.</t>
         </is>
       </c>
     </row>
@@ -2130,37 +2755,52 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
           <t>TC-042</t>
         </is>
       </c>
-      <c r="C46" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E46" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>failed (крок 3)</t>
-        </is>
-      </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H46" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 5)</t>
+        </is>
+      </c>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
           <t>BUG-010 (#33)</t>
         </is>
       </c>
-      <c r="H46" s="4" t="inlineStr">
-        <is>
-          <t>У режимі Edit немає стовпця Total і підсумкового рядка; після Tab підсумки не з'являються. Cancel.</t>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: виконано під Admin замість qp.ess.ivan, тиждень і активність не з кейсу.</t>
         </is>
       </c>
     </row>
@@ -2172,31 +2812,46 @@
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
           <t>TC-043</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>15:14</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr"/>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
         <is>
           <t>QP Test Vacancy (Active) у списку і в Vacancy форми кандидата; видалено.</t>
         </is>
@@ -2210,33 +2865,48 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
           <t>TC-044</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>15:14</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>Qpkand Kandydatenko з qp_resume.pdf: Application Initiated, кнопки Reject / Shortlist; видалено.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I48" s="4" t="inlineStr"/>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: кандидат Qptest Candidate замість Qpkand Kandydatenko з кейсу.</t>
         </is>
       </c>
     </row>
@@ -2248,31 +2918,46 @@
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
           <t>TC-045</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E49" s="4" t="inlineStr">
+        <is>
+          <t>15:16</t>
+        </is>
+      </c>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr"/>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
         <is>
           <t>Поля форми за GUI-90; підказка «Accepts .docx, .doc, .odt, .pdf, .rtf, .txt up to 1MB».</t>
         </is>
@@ -2286,31 +2971,46 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
           <t>TC-046</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E50" s="4" t="inlineStr">
+        <is>
+          <t>15:16</t>
+        </is>
+      </c>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H50" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I50" s="4" t="inlineStr"/>
+      <c r="J50" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K50" s="4" t="inlineStr">
         <is>
           <t>«File type not allowed» для qp_resume.png; кандидата не збережено.</t>
         </is>
@@ -2324,31 +3024,46 @@
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
           <t>TC-047</t>
         </is>
       </c>
-      <c r="C51" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E51" s="4" t="inlineStr">
+        <is>
+          <t>15:16</t>
+        </is>
+      </c>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E51" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G51" s="4" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr"/>
+      <c r="J51" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K51" s="4" t="inlineStr">
         <is>
           <t>«Attachment Size Exceeded» для qp_big.pdf (1 200 000 байт); кандидата не збережено.</t>
         </is>
@@ -2362,37 +3077,52 @@
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
           <t>TC-048</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E52" s="4" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H52" s="4" t="inlineStr">
         <is>
           <t>failed (крок 4)</t>
         </is>
       </c>
-      <c r="G52" s="4" t="inlineStr">
+      <c r="I52" s="4" t="inlineStr">
         <is>
           <t>BUG-011 (#34)</t>
         </is>
       </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>Повідомлення про формат немає; кандидата Qpmail збережено з qp.kand@example.c і видалено очищенням.</t>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K52" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: email qptest@example.c замість qp.kand@example.c з кейсу.</t>
         </is>
       </c>
     </row>
@@ -2404,33 +3134,48 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
           <t>TC-049</t>
         </is>
       </c>
-      <c r="C53" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E53" s="4" t="inlineStr">
+        <is>
+          <t>15:14</t>
+        </is>
+      </c>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E53" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>passed</t>
-        </is>
-      </c>
-      <c r="G53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
       <c r="H53" s="4" t="inlineStr">
         <is>
-          <t>qp.kand@example.ua прийнято без повідомлень; кандидата збережено і видалено.</t>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr"/>
+      <c r="J53" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K53" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: email qptest@example.ua замість qp.kand@example.ua з кейсу.</t>
         </is>
       </c>
     </row>
@@ -2442,42 +3187,1369 @@
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
           <t>TC-050</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
-        <is>
-          <t>27.10.2026</t>
-        </is>
-      </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E54" s="4" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
           <t>Шпилька Т.</t>
         </is>
       </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H54" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I54" s="4" t="inlineStr"/>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 2</t>
+        </is>
+      </c>
+      <c r="K54" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: очікуване переписано під фактичне (довідка англійською), крок 3 виконано не зі сторінки PIM; статус passed хибний.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>TC-001</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E55" s="4" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr"/>
+      <c r="J55" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K55" s="4" t="inlineStr">
+        <is>
+          <t>Dashboard; меню з 12 пунктів: Admin, PIM, Leave, Time, Recruitment, My Info, Performance, Dashboard, Directory, Maintenance, Claim, Buzz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>TC-014</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E56" s="4" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H56" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 9)</t>
+        </is>
+      </c>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>BUG-003 (#25)</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K56" s="4" t="inlineStr">
+        <is>
+          <t>Повідомлення про 8 символів немає (індикатор «Better»); на кроці 10 користувача збережено і видалено очищенням.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>TC-015</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E57" s="4" t="inlineStr">
+        <is>
+          <t>16:16</t>
+        </is>
+      </c>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 9)</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>BUG-004 (#26)</t>
+        </is>
+      </c>
+      <c r="J57" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K57" s="4" t="inlineStr">
+        <is>
+          <t>Повідомлення про велику літеру немає (індикатор «Strong»); користувача збережено і видалено очищенням.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>TC-016</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>16:18</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 9)</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>BUG-005 (#27)</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>Повідомлення про спецсимвол немає (індикатор «Weak»); користувача збережено і видалено очищенням.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>TC-018</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Мініцька А.</t>
+        </is>
+      </c>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr"/>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K59" s="4" t="inlineStr">
+        <is>
+          <t>Стовпці і фільтри за F-40; Include: Current Employees Only / Current and Past Employees / Past Employees Only; пошук за Id — (1) Record Found.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>TC-021</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E60" s="4" t="inlineStr">
+        <is>
+          <t>16:22</t>
+        </is>
+      </c>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Мініцька А.</t>
+        </is>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H60" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 7)</t>
+        </is>
+      </c>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>BUG-006 (#28)</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K60" s="4" t="inlineStr">
+        <is>
+          <t>«Success / Successfully Saved» ліворуч унизу замість праворуч; запропонований Employee Id записано; Qpanna видалено.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>TC-026</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E61" s="4" t="inlineStr">
+        <is>
+          <t>16:26</t>
+        </is>
+      </c>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Мініцька А.</t>
+        </is>
+      </c>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr"/>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор вручну</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>Не зараховано: час виміряно через performance.getEntriesByType('navigation')[0].duration (лише HTML-документ, без завантаження даних сторінки), а не Finish у DevTools → Network, як вимагає кейс; p95 = 1,32 с.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>TC-029</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>16:28</t>
+        </is>
+      </c>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H62" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 5)</t>
+        </is>
+      </c>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>— (дефект кейсу)</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>ні — повтор у проході 3</t>
+        </is>
+      </c>
+      <c r="K62" s="4" t="inlineStr">
+        <is>
+          <t>Версія кейсу 1.0. Дефект тест-кейсу: очікуване «Partial Days зі значенням None» не випливає з GUI-70 (фактично «-- Select --», список є). Кейс виправлено до v1.1 (аркуш Review), баг-репорт не заводиться; повтор — прохід 3.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>TC-031</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>16:33</t>
+        </is>
+      </c>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 8)</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>BUG-009 (#32)</t>
+        </is>
+      </c>
+      <c r="J63" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>Number of Days 3.00 замість 5.00 — свята 11.11 і 12.11 вилучено. Заявку скасовано.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>TC-033</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E64" s="4" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H64" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I64" s="4" t="inlineStr"/>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>«Balance not sufficient»; після Apply тост «Leave Balance Exceeded»; заявки немає в My Leave.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>TC-034</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E65" s="4" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I65" s="4" t="inlineStr"/>
+      <c r="J65" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K65" s="4" t="inlineStr">
+        <is>
+          <t>16–20.11 = 5.00 при балансі 5.00: «Successfully Saved», Pending Approval (5.00); скасовано.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>TC-035</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E66" s="4" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H66" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I66" s="4" t="inlineStr"/>
+      <c r="J66" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
+          <t>Заявку 17.11 скасовано: Cancelled (1.00), баланс знову 5.00; фільтр статусів — 5 варіантів.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>TC-036</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E67" s="4" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr"/>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>Заявка 18.11 відхилена Admin: Rejected (1.00), кнопки Cancel у ESS немає.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>TC-037</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H68" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I68" s="4" t="inlineStr"/>
+      <c r="J68" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t>My Actions «(1) Leave Requests to Approve»; Approve → Scheduled (1.00); скасовано очищенням.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>TC-040</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Шпилька Т.</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr"/>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>Табель 26.10–01.11, ACME Ltd / Bug Fixes, 8:00: Save → Not Submitted, Submit → Submitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>TC-041</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="inlineStr">
+        <is>
+          <t>17:02</t>
+        </is>
+      </c>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Шпилька Т.</t>
+        </is>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H70" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I70" s="4" t="inlineStr"/>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>Табель 19.10–25.10 подано (Submitted) і затверджено Admin з коментарем QP TC-041 (Approved).</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>TC-042</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E71" s="4" t="inlineStr">
+        <is>
+          <t>17:09</t>
+        </is>
+      </c>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>Шпилька Т.</t>
+        </is>
+      </c>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 3)</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>BUG-010 (#33)</t>
+        </is>
+      </c>
+      <c r="J71" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K71" s="4" t="inlineStr">
+        <is>
+          <t>У режимі Edit немає стовпця Total і підсумкового рядка; після Tab підсумки не з'являються. Cancel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>TC-044</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>17:11</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>Шпилька Т.</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I72" s="4" t="inlineStr"/>
+      <c r="J72" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K72" s="4" t="inlineStr">
+        <is>
+          <t>Qpkand Kandydatenko з qp_resume.pdf: Application Initiated, кнопки Reject / Shortlist; видалено.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>TC-048</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>17:13</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>Шпилька Т.</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
         <is>
           <t>failed (крок 4)</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr">
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>BUG-011 (#34)</t>
+        </is>
+      </c>
+      <c r="J73" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K73" s="4" t="inlineStr">
+        <is>
+          <t>Повідомлення про формат немає; кандидата Qpmail збережено з qp.kand@example.c і видалено очищенням.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>TC-049</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>17:16</t>
+        </is>
+      </c>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>Шпилька Т.</t>
+        </is>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H74" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I74" s="4" t="inlineStr"/>
+      <c r="J74" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K74" s="4" t="inlineStr">
+        <is>
+          <t>qp.kand@example.ua прийнято без повідомлень; кандидата збережено і видалено.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>TC-050</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E75" s="4" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>Шпилька Т.</t>
+        </is>
+      </c>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 4)</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="inlineStr">
         <is>
           <t>BUG-012 (#35)</t>
         </is>
       </c>
-      <c r="H54" s="4" t="inlineStr">
+      <c r="J75" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K75" s="4" t="inlineStr">
         <is>
           <t>Відкрито англомовний starterhelp.orangehrm.com/hc/en-us; структури D-10 немає.</t>
         </is>
       </c>
     </row>
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>TC-008</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H76" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 5)</t>
+        </is>
+      </c>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>BUG-002 (#24)</t>
+        </is>
+      </c>
+      <c r="J76" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K76" s="4" t="inlineStr">
+        <is>
+          <t>Після 16 хв 19 с бездіяльності (20:46:28–21:02:47) Leave List відкрився без входу. Відтворено у двох сеансах.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>ручний</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>TC-026</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>27.10.2026</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>22:01</t>
+        </is>
+      </c>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>Шпилька Т.</t>
+        </is>
+      </c>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>failed (крок 7)</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>BUG-008 (#31)</t>
+        </is>
+      </c>
+      <c r="J77" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K77" s="4" t="inlineStr">
+        <is>
+          <t>p95 = 6,48 с (10 з 20 &gt; 3 с). Відхилення: 4-та сторінка — Admin → User Management замість Recruitment → Vacancies (без неї 7 з 15 &gt; 3 с); швидкість каналу виміряно не перед замірами, а 28.10.2026 з того самого підключення: fast.com — 910 Мбіт/с (≥ 10 за передумовою).</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
+        <is>
+          <t>Run 1</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>TC-029</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>28.10.2026</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="inlineStr">
+        <is>
+          <t>12:20</t>
+        </is>
+      </c>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Любочка В.</t>
+        </is>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>E1: demo OrangeHRM OS 5.9; Chrome 155, Windows 11</t>
+        </is>
+      </c>
+      <c r="H78" s="4" t="inlineStr">
+        <is>
+          <t>passed</t>
+        </is>
+      </c>
+      <c r="I78" s="4" t="inlineStr"/>
+      <c r="J78" s="4" t="inlineStr">
+        <is>
+          <t>так</t>
+        </is>
+      </c>
+      <c r="K78" s="4" t="inlineStr">
+        <is>
+          <t>Виконано за версією кейсу 1.1 (прохід 3): після введення дат показано список Partial Days. Версія 1.0 у проході 2 дала хибний failed через помилку в очікуваному (аркуш Review).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:H54"/>
+  <autoFilter ref="A4:K78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2488,7 +4560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2620,101 +4692,113 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Тестові дані (SETUP-1)</t>
+          <t>Рядки журналу</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Qpivan Testenko (Employee Id 0370 у проході 2; 0373 у проході 1), користувач qp.ess.ivan / QpTest#2026; Qpolha Vymknena, користувач qp.ess.off (Disabled); ліміт US - Vacation 5.00</t>
+          <t>74 виконання: прохід 1 — 50, прохід 2 — 22, TC-026 вручну — 1, прохід 3 — 1. Зараховано 50 (останнє виконання кожного кейсу, стовпець «Зараховано»); попередні виконання лишаються в журналі з причиною повтору</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Свята demo (листопад 2026)</t>
+          <t>Тестові дані (SETUP-1)</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>2026-11-11 Remembrance Day (Canada) — Full Day; 2026-12-11 (12.11) Veterans Day (US) — Full Day</t>
+          <t>Qpivan Testenko (Employee Id 0370 у проході 2; 0373 у проході 1), користувач qp.ess.ivan / QpTest#2026; Qpolha Vymknena, користувач qp.ess.off (Disabled); ліміт US - Vacation 5.00</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Тестові файли</t>
+          <t>Свята demo (листопад 2026)</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>qp_resume.pdf (1 947 Б), qp_resume.png (6 401 Б), qp_big.pdf (1 200 000 Б)</t>
+          <t>2026-11-11 Remembrance Day (Canada) — Full Day; 2026-12-11 (12.11) Veterans Day (US) — Full Day</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Прохід 3</t>
+          <t>Тестові файли</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>28.10.2026, 12:10–12:26: TC-029 за версією кейсу 1.1 (після рецензування результату проходу 2); SETUP-1 повторено (Qpivan Testenko — Employee Id 0422), скидань demo не було, TEARDOWN-1 виконано</t>
+          <t>qp_resume.pdf (1 947 Б), qp_resume.png (6 401 Б), qp_big.pdf (1 200 000 Б)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Скидання demo</t>
+          <t>Прохід 3</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Прохід 1: ~14:00 дані SETUP-1 зникли, SETUP-1 повторено. Прохід 2: скидань не було.</t>
+          <t>28.10.2026, 12:10–12:26: TC-029 за версією кейсу 1.1 (після рецензування результату проходу 2); SETUP-1 повторено (Qpivan Testenko — Employee Id 0422), скидань demo не було, TEARDOWN-1 виконано</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>TEARDOWN-1</t>
+          <t>Скидання demo</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Виконано після кожного проходу: записи з префіксом Qp / qp. видалено</t>
+          <t>Прохід 1: ~14:00 дані SETUP-1 зникли, SETUP-1 повторено. Прохід 2: скидань не було.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>TC-026 (P-10)</t>
+          <t>TEARDOWN-1</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>DevTools → Network, Disable cache, No throttling; Finish для 20 переходів (27.10.2026, 22:01–22:04). Швидкість каналу: fast.com — 910 Мбіт/с, виміряно 28.10.2026 з того самого підключення (не перед замірами — відхилення від передумов кейсу)</t>
+          <t>Виконано після кожного проходу: записи з префіксом Qp / qp. видалено</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
+          <t>TC-026 (P-10)</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>DevTools → Network, Disable cache, No throttling; Finish для 20 переходів (27.10.2026, 22:01–22:04). Швидкість каналу: fast.com — 910 Мбіт/с, виміряно 28.10.2026 з того самого підключення (не перед замірами — відхилення від передумов кейсу)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>Стан demo, що впливав на прогін</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Спільні дані змінюються іншими користувачами: перейменовано працівника Admin («john Doe», «ana yaa»), змінено колірну тему і період відпусток (2026-01-01 – 2027-03-03)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B20"/>
+  <autoFilter ref="A4:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>